<commit_message>
I may have made too many changes
</commit_message>
<xml_diff>
--- a/study_case_model/bigger_network/scenario_variables/demand_scenarios152.xlsx
+++ b/study_case_model/bigger_network/scenario_variables/demand_scenarios152.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>14362.67807379212</v>
+        <v>1034.112821313033</v>
       </c>
     </row>
     <row r="3">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>14362.67807379212</v>
+        <v>114.901424590337</v>
       </c>
     </row>
     <row r="4">
@@ -527,16 +527,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>958.5207096486446</v>
       </c>
     </row>
     <row r="6">
@@ -553,11 +553,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>14377.81064472967</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -574,7 +574,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -590,16 +590,16 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>4792.603548243223</v>
+        <v>955.4452491441662</v>
       </c>
     </row>
     <row r="9">
@@ -611,16 +611,16 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4792.603548243223</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -632,16 +632,16 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>59715.32807151039</v>
+        <v>238.8613122860415</v>
       </c>
     </row>
     <row r="11">
@@ -658,11 +658,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1456.908956922408</v>
       </c>
     </row>
     <row r="12">
@@ -679,7 +679,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -700,7 +700,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>18211.3619615301</v>
+        <v>929.7539875829992</v>
       </c>
     </row>
     <row r="15">
@@ -775,20 +775,20 @@
         <v>2</v>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>836.7830216237212</v>
       </c>
     </row>
     <row r="18">
@@ -805,11 +805,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>11621.92484478749</v>
+        <v>92.97589129152459</v>
       </c>
     </row>
     <row r="19">
@@ -826,11 +826,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>11621.92484478749</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -842,16 +842,16 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1473.763844652217</v>
       </c>
     </row>
     <row r="21">
@@ -863,12 +863,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -889,11 +889,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>13946.38369372869</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -905,16 +905,16 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>984.1843349966981</v>
       </c>
     </row>
     <row r="24">
@@ -926,16 +926,16 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>4648.794564576229</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -947,16 +947,16 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>4648.794564576229</v>
+        <v>246.0460837491745</v>
       </c>
     </row>
     <row r="26">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>73688.19223261088</v>
+        <v>859.1576842195143</v>
       </c>
     </row>
     <row r="27">
@@ -1031,16 +1031,16 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>1162.768013075789</v>
       </c>
     </row>
     <row r="30">
@@ -1057,11 +1057,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>15377.88023432341</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -1090,20 +1090,20 @@
         <v>2</v>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>774.8772229406352</v>
       </c>
     </row>
     <row r="33">
@@ -1111,20 +1111,20 @@
         <v>2</v>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>86.09746921562613</v>
       </c>
     </row>
     <row r="34">
@@ -1141,11 +1141,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>10739.47105274393</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1157,16 +1157,16 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>10739.47105274393</v>
+        <v>860.281073928923</v>
       </c>
     </row>
     <row r="36">
@@ -1178,12 +1178,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -1199,12 +1199,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>17441.52019613684</v>
+        <v>858.0709451758481</v>
       </c>
     </row>
     <row r="39">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>5813.840065378947</v>
+        <v>214.517736293962</v>
       </c>
     </row>
     <row r="41">
@@ -1283,16 +1283,16 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>5813.840065378947</v>
+        <v>426.0159266026606</v>
       </c>
     </row>
     <row r="42">
@@ -1309,11 +1309,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>43048.73460781306</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -1346,16 +1346,16 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0</v>
+        <v>482.5246502460902</v>
       </c>
     </row>
     <row r="45">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -1393,11 +1393,11 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>10753.51342411154</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1405,20 +1405,20 @@
         <v>2</v>
       </c>
       <c r="B47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>748.1823671049374</v>
       </c>
     </row>
     <row r="48">
@@ -1426,20 +1426,20 @@
         <v>2</v>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>83.13137412277082</v>
       </c>
     </row>
     <row r="49">
@@ -1447,16 +1447,16 @@
         <v>2</v>
       </c>
       <c r="B49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>13407.35851837263</v>
+        <v>696.1506638996728</v>
       </c>
     </row>
     <row r="51">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1502,7 +1502,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>13407.35851837263</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1535,16 +1535,16 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>875.4193598228657</v>
       </c>
     </row>
     <row r="54">
@@ -1556,16 +1556,16 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>6390.238899039909</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -1577,16 +1577,16 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0</v>
+        <v>218.8548399557164</v>
       </c>
     </row>
     <row r="56">
@@ -1598,16 +1598,16 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>2130.079633013303</v>
+        <v>727.5927773436368</v>
       </c>
     </row>
     <row r="57">
@@ -1619,16 +1619,16 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>2130.079633013303</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -1645,11 +1645,11 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>24126.23251230451</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -1661,16 +1661,16 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0</v>
+        <v>576.3088895994126</v>
       </c>
     </row>
     <row r="60">
@@ -1682,12 +1682,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -1703,12 +1703,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -1720,11 +1720,11 @@
         <v>2</v>
       </c>
       <c r="B62" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>10391.42176534635</v>
+        <v>1295.72516760882</v>
       </c>
     </row>
     <row r="63">
@@ -1741,11 +1741,11 @@
         <v>2</v>
       </c>
       <c r="B63" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1754,7 +1754,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0</v>
+        <v>143.9694630676466</v>
       </c>
     </row>
     <row r="64">
@@ -1762,11 +1762,11 @@
         <v>2</v>
       </c>
       <c r="B64" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1783,20 +1783,20 @@
         <v>2</v>
       </c>
       <c r="B65" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0</v>
+        <v>932.2671098540393</v>
       </c>
     </row>
     <row r="66">
@@ -1808,16 +1808,16 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>8701.88329874591</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -1829,16 +1829,16 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>8701.88329874591</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -1850,16 +1850,16 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0</v>
+        <v>816.2067691251018</v>
       </c>
     </row>
     <row r="69">
@@ -1871,12 +1871,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -1892,16 +1892,16 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Equinor Energy AS</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>16414.11299667873</v>
+        <v>204.0516922812755</v>
       </c>
     </row>
     <row r="71">
@@ -1913,16 +1913,16 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>Equinor Energy AS</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0</v>
+        <v>572.575544135963</v>
       </c>
     </row>
     <row r="72">
@@ -1934,16 +1934,16 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Vår Energi ASA</t>
+          <t>SHELL</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>5471.370998892911</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -1955,16 +1955,16 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Aker BP ASA</t>
+          <t>Vår Energi ASA</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>5471.370998892911</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>36379.63886718184</v>
+        <v>836.6851826424452</v>
       </c>
     </row>
     <row r="75">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2027,111 +2027,6 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="n">
-        <v>2</v>
-      </c>
-      <c r="B77" t="n">
-        <v>5</v>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>DUNKERQUE</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Aker BP ASA</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>2</v>
-      </c>
-      <c r="B78" t="n">
-        <v>5</v>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>EASINGTON</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Equinor Energy AS</t>
-        </is>
-      </c>
-      <c r="E78" t="n">
-        <v>7203.861119992658</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>2</v>
-      </c>
-      <c r="B79" t="n">
-        <v>5</v>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>EASINGTON</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>SHELL</t>
-        </is>
-      </c>
-      <c r="E79" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>2</v>
-      </c>
-      <c r="B80" t="n">
-        <v>5</v>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>EASINGTON</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Vår Energi ASA</t>
-        </is>
-      </c>
-      <c r="E80" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>2</v>
-      </c>
-      <c r="B81" t="n">
-        <v>5</v>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>EASINGTON</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Aker BP ASA</t>
-        </is>
-      </c>
-      <c r="E81" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>